<commit_message>
Add reproducible benchmark scaffold + Claude baseline run
- Prompt (prompts/factcheck_prompt_kk.txt), blind multi-provider runner,
  scoring (accuracy/macro-F1/kappa/confusion), dataset export and source
  extraction scripts
- Model registry (scripts/models.json); keys read from .env only, .env
  git-ignored (.env.example template committed)
- Git-diffable dataset mirrors (data/dataset.csv|.jsonl) and versioned
  source text (sources/leg_text01.txt)
- Claude blind baseline recorded (results/claude_blind_run.json, 19/20);
  claude_label written into dataset
- README documents method, taxonomy, run protocol

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -474,7 +474,11 @@
       <c r="H2" s="4" t="n"/>
       <c r="I2" s="4" t="n"/>
       <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="L2" s="4" t="n"/>
       <c r="M2" s="4" t="n"/>
       <c r="N2" s="4" t="n"/>
@@ -530,7 +534,11 @@
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="4" t="n"/>
       <c r="J3" s="4" t="n"/>
-      <c r="K3" s="4" t="n"/>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="L3" s="4" t="n"/>
       <c r="M3" s="4" t="n"/>
       <c r="N3" s="4" t="n"/>
@@ -586,7 +594,11 @@
       <c r="H4" s="4" t="n"/>
       <c r="I4" s="4" t="n"/>
       <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="L4" s="4" t="n"/>
       <c r="M4" s="4" t="n"/>
       <c r="N4" s="4" t="n"/>
@@ -642,7 +654,11 @@
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="n"/>
       <c r="J5" s="4" t="n"/>
-      <c r="K5" s="4" t="n"/>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="L5" s="4" t="n"/>
       <c r="M5" s="4" t="n"/>
       <c r="N5" s="4" t="n"/>
@@ -698,7 +714,11 @@
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="4" t="n"/>
-      <c r="K6" s="4" t="n"/>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="L6" s="4" t="n"/>
       <c r="M6" s="4" t="n"/>
       <c r="N6" s="4" t="n"/>
@@ -754,7 +774,11 @@
       <c r="H7" s="4" t="n"/>
       <c r="I7" s="4" t="n"/>
       <c r="J7" s="4" t="n"/>
-      <c r="K7" s="4" t="n"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="L7" s="4" t="n"/>
       <c r="M7" s="4" t="n"/>
       <c r="N7" s="4" t="n"/>
@@ -810,7 +834,11 @@
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="4" t="n"/>
       <c r="J8" s="4" t="n"/>
-      <c r="K8" s="4" t="n"/>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="L8" s="4" t="n"/>
       <c r="M8" s="4" t="n"/>
       <c r="N8" s="4" t="n"/>
@@ -866,7 +894,11 @@
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="4" t="n"/>
       <c r="J9" s="4" t="n"/>
-      <c r="K9" s="4" t="n"/>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="L9" s="4" t="n"/>
       <c r="M9" s="4" t="n"/>
       <c r="N9" s="4" t="n"/>
@@ -922,7 +954,11 @@
       <c r="H10" s="4" t="n"/>
       <c r="I10" s="4" t="n"/>
       <c r="J10" s="4" t="n"/>
-      <c r="K10" s="4" t="n"/>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="L10" s="4" t="n"/>
       <c r="M10" s="4" t="n"/>
       <c r="N10" s="4" t="n"/>
@@ -978,7 +1014,11 @@
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="4" t="n"/>
       <c r="J11" s="4" t="n"/>
-      <c r="K11" s="4" t="n"/>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="L11" s="4" t="n"/>
       <c r="M11" s="4" t="n"/>
       <c r="N11" s="4" t="n"/>
@@ -1034,7 +1074,11 @@
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="4" t="n"/>
       <c r="J12" s="4" t="n"/>
-      <c r="K12" s="4" t="n"/>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="L12" s="4" t="n"/>
       <c r="M12" s="4" t="n"/>
       <c r="N12" s="4" t="n"/>
@@ -1090,7 +1134,11 @@
       <c r="H13" s="4" t="n"/>
       <c r="I13" s="4" t="n"/>
       <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="n"/>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="L13" s="4" t="n"/>
       <c r="M13" s="4" t="n"/>
       <c r="N13" s="4" t="n"/>
@@ -1146,7 +1194,11 @@
       <c r="H14" s="4" t="n"/>
       <c r="I14" s="4" t="n"/>
       <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="n"/>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="L14" s="4" t="n"/>
       <c r="M14" s="4" t="n"/>
       <c r="N14" s="4" t="n"/>
@@ -1202,7 +1254,11 @@
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="4" t="n"/>
       <c r="J15" s="4" t="n"/>
-      <c r="K15" s="4" t="n"/>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="L15" s="4" t="n"/>
       <c r="M15" s="4" t="n"/>
       <c r="N15" s="4" t="n"/>
@@ -1258,7 +1314,11 @@
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="4" t="n"/>
       <c r="J16" s="4" t="n"/>
-      <c r="K16" s="4" t="n"/>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="L16" s="4" t="n"/>
       <c r="M16" s="4" t="n"/>
       <c r="N16" s="4" t="n"/>
@@ -1314,7 +1374,11 @@
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="4" t="n"/>
       <c r="J17" s="4" t="n"/>
-      <c r="K17" s="4" t="n"/>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="L17" s="4" t="n"/>
       <c r="M17" s="4" t="n"/>
       <c r="N17" s="4" t="n"/>
@@ -1370,7 +1434,11 @@
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="4" t="n"/>
       <c r="J18" s="4" t="n"/>
-      <c r="K18" s="4" t="n"/>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="L18" s="4" t="n"/>
       <c r="M18" s="4" t="n"/>
       <c r="N18" s="4" t="n"/>
@@ -1427,7 +1495,11 @@
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="4" t="n"/>
       <c r="J19" s="4" t="n"/>
-      <c r="K19" s="4" t="n"/>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="L19" s="4" t="n"/>
       <c r="M19" s="4" t="n"/>
       <c r="N19" s="4" t="n"/>
@@ -1484,7 +1556,11 @@
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="4" t="n"/>
       <c r="J20" s="4" t="n"/>
-      <c r="K20" s="4" t="n"/>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="L20" s="4" t="n"/>
       <c r="M20" s="4" t="n"/>
       <c r="N20" s="4" t="n"/>
@@ -1540,7 +1616,11 @@
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="4" t="n"/>
       <c r="J21" s="4" t="n"/>
-      <c r="K21" s="4" t="n"/>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="L21" s="4" t="n"/>
       <c r="M21" s="4" t="n"/>
       <c r="N21" s="4" t="n"/>

</xml_diff>

<commit_message>
Add Gemini 2.5 Flash run results (19/20) and gemini_label
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -471,7 +471,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H2" s="4" t="n"/>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I2" s="4" t="n"/>
       <c r="J2" s="4" t="n"/>
       <c r="K2" s="4" t="inlineStr">
@@ -531,7 +535,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H3" s="4" t="n"/>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I3" s="4" t="n"/>
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="inlineStr">
@@ -591,7 +599,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H4" s="4" t="n"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I4" s="4" t="n"/>
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="inlineStr">
@@ -651,7 +663,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H5" s="4" t="n"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I5" s="4" t="n"/>
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="4" t="inlineStr">
@@ -711,7 +727,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="H6" s="4" t="n"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="4" t="n"/>
       <c r="K6" s="4" t="inlineStr">
@@ -771,7 +791,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H7" s="4" t="n"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I7" s="4" t="n"/>
       <c r="J7" s="4" t="n"/>
       <c r="K7" s="4" t="inlineStr">
@@ -831,7 +855,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H8" s="4" t="n"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I8" s="4" t="n"/>
       <c r="J8" s="4" t="n"/>
       <c r="K8" s="4" t="inlineStr">
@@ -891,7 +919,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H9" s="4" t="n"/>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I9" s="4" t="n"/>
       <c r="J9" s="4" t="n"/>
       <c r="K9" s="4" t="inlineStr">
@@ -951,7 +983,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="H10" s="4" t="n"/>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I10" s="4" t="n"/>
       <c r="J10" s="4" t="n"/>
       <c r="K10" s="4" t="inlineStr">
@@ -1011,7 +1047,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H11" s="4" t="n"/>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I11" s="4" t="n"/>
       <c r="J11" s="4" t="n"/>
       <c r="K11" s="4" t="inlineStr">
@@ -1071,7 +1111,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H12" s="4" t="n"/>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I12" s="4" t="n"/>
       <c r="J12" s="4" t="n"/>
       <c r="K12" s="4" t="inlineStr">
@@ -1131,7 +1175,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H13" s="4" t="n"/>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I13" s="4" t="n"/>
       <c r="J13" s="4" t="n"/>
       <c r="K13" s="4" t="inlineStr">
@@ -1191,7 +1239,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H14" s="4" t="n"/>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I14" s="4" t="n"/>
       <c r="J14" s="4" t="n"/>
       <c r="K14" s="4" t="inlineStr">
@@ -1251,7 +1303,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H15" s="4" t="n"/>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I15" s="4" t="n"/>
       <c r="J15" s="4" t="n"/>
       <c r="K15" s="4" t="inlineStr">
@@ -1311,7 +1367,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H16" s="4" t="n"/>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I16" s="4" t="n"/>
       <c r="J16" s="4" t="n"/>
       <c r="K16" s="4" t="inlineStr">
@@ -1371,7 +1431,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H17" s="4" t="n"/>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I17" s="4" t="n"/>
       <c r="J17" s="4" t="n"/>
       <c r="K17" s="4" t="inlineStr">
@@ -1431,7 +1495,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H18" s="4" t="n"/>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I18" s="4" t="n"/>
       <c r="J18" s="4" t="n"/>
       <c r="K18" s="4" t="inlineStr">
@@ -1492,7 +1560,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H19" s="4" t="n"/>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I19" s="4" t="n"/>
       <c r="J19" s="4" t="n"/>
       <c r="K19" s="4" t="inlineStr">
@@ -1553,7 +1625,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H20" s="4" t="n"/>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I20" s="4" t="n"/>
       <c r="J20" s="4" t="n"/>
       <c r="K20" s="4" t="inlineStr">
@@ -1613,7 +1689,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="H21" s="4" t="n"/>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I21" s="4" t="n"/>
       <c r="J21" s="4" t="n"/>
       <c r="K21" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add DeepSeek run (18/20) and deepseek_label
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -420,7 +420,7 @@
           <t>kimi_label</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="0" t="inlineStr">
         <is>
           <t>qwen_label</t>
         </is>
@@ -487,7 +487,11 @@
         </is>
       </c>
       <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -498,7 +502,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -561,7 +565,11 @@
         </is>
       </c>
       <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="n"/>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -572,7 +580,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M3" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -635,7 +643,11 @@
         </is>
       </c>
       <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="n"/>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -646,7 +658,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -709,7 +721,11 @@
         </is>
       </c>
       <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="n"/>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -720,7 +736,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M5" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -783,7 +799,11 @@
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
-      <c r="J6" s="4" t="n"/>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -794,7 +814,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M6" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -857,7 +877,11 @@
         </is>
       </c>
       <c r="I7" s="4" t="n"/>
-      <c r="J7" s="4" t="n"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -868,7 +892,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M7" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -931,7 +955,11 @@
         </is>
       </c>
       <c r="I8" s="4" t="n"/>
-      <c r="J8" s="4" t="n"/>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -942,7 +970,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M8" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -1005,7 +1033,11 @@
         </is>
       </c>
       <c r="I9" s="4" t="n"/>
-      <c r="J9" s="4" t="n"/>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -1016,7 +1048,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M9" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -1079,7 +1111,11 @@
         </is>
       </c>
       <c r="I10" s="4" t="n"/>
-      <c r="J10" s="4" t="n"/>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -1090,7 +1126,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M10" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -1153,7 +1189,11 @@
         </is>
       </c>
       <c r="I11" s="4" t="n"/>
-      <c r="J11" s="4" t="n"/>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -1164,7 +1204,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M11" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -1227,7 +1267,11 @@
         </is>
       </c>
       <c r="I12" s="4" t="n"/>
-      <c r="J12" s="4" t="n"/>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -1238,7 +1282,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M12" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -1301,7 +1345,11 @@
         </is>
       </c>
       <c r="I13" s="4" t="n"/>
-      <c r="J13" s="4" t="n"/>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -1312,7 +1360,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M13" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -1375,7 +1423,11 @@
         </is>
       </c>
       <c r="I14" s="4" t="n"/>
-      <c r="J14" s="4" t="n"/>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -1386,7 +1438,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M14" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -1449,7 +1501,11 @@
         </is>
       </c>
       <c r="I15" s="4" t="n"/>
-      <c r="J15" s="4" t="n"/>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -1460,7 +1516,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M15" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -1523,7 +1579,11 @@
         </is>
       </c>
       <c r="I16" s="4" t="n"/>
-      <c r="J16" s="4" t="n"/>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -1534,7 +1594,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M16" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -1597,7 +1657,11 @@
         </is>
       </c>
       <c r="I17" s="4" t="n"/>
-      <c r="J17" s="4" t="n"/>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -1608,7 +1672,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M17" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -1671,7 +1735,11 @@
         </is>
       </c>
       <c r="I18" s="4" t="n"/>
-      <c r="J18" s="4" t="n"/>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -1682,7 +1750,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M18" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -1746,7 +1814,11 @@
         </is>
       </c>
       <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="n"/>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -1757,7 +1829,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M19" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -1821,7 +1893,11 @@
         </is>
       </c>
       <c r="I20" s="4" t="n"/>
-      <c r="J20" s="4" t="n"/>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -1832,7 +1908,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M20" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -1895,7 +1971,11 @@
         </is>
       </c>
       <c r="I21" s="4" t="n"/>
-      <c r="J21" s="4" t="n"/>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -1906,7 +1986,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M21" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>

</xml_diff>

<commit_message>
Add source text 2 (news_text1): 21 claims (021-041)
- append news_text1 rows to dataset (kept text-1 with fixes/labels intact)
- sources/news_text1.txt extracted; prompts/chat_run_news_text1.txt generated
- score.py filters gold by the run's source_doc (multi-source aware)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -2008,13 +2008,42 @@
       <c r="AB21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>021</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026 жылғы 13 шілдеде мемлекет басшысы Премьер-министр Олжас Бектеновті қабылдады. Қасым-Жомарт Тоқаев Қазақстан Республикасының биылғы қаңтар-маусым айларындағы әлеуметтік-экономикалық даму қорытындылары туралы есепті тыңдап, экономиканы одан әрі әртараптандыру жоспарымен танысты.
+</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Тоқаев Бектеновпен 2 маусымда кездесті.</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>fake_entity</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026 жылғы 13 шілдеде мемлекет басшысы Премьер-министр Олжас Бектеновті қабылдады. </t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="4" t="n"/>
       <c r="J22" s="4" t="n"/>
@@ -2036,13 +2065,41 @@
       <c r="AB22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n"/>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>022</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Премьер-министр бірінші жартыжылдық қорытындысы бойынша ішкі жалпы өнім көлемі 4,1 пайызға өскенін баяндады. </t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Бірінші жартыжылдық қорытындысы бойынша ішкі жалпы өнім өспеді.</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>fake_entity</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Премьер-министр бірінші жартыжылдық қорытындысы бойынша ішкі жалпы өнім көлемі 4,1 пайызға өскенін баяндады. </t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
       <c r="J23" s="4" t="n"/>
@@ -2064,13 +2121,41 @@
       <c r="AB23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n"/>
-      <c r="B24" s="4" t="n"/>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
-      <c r="G24" s="4" t="n"/>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>023</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Премьер-министр бірінші жартыжылдық қорытындысы бойынша ішкі жалпы өнім көлемі 4,1 пайызға өскенін баяндады. Экономика құрылымындағы өңдеу өнеркәсібінің үлесі – 9,8 пайызға, көлік саласы – 7,1 пайызға, құрылыс 15,2 пайызға артты. Сондай-ақ сауда-саттықта – 5,7 пайыз, ауыл шаруашылығында – 4,4 пайыз және байланыс қызметінде 4,3 пайыз өсім тіркелді. Негізгі капиталға тартылған инвестиция көлемі 9,5 триллион теңгені құрады, соның ішінде жеке инвестиция 21,4 пайызға ұлғайды.</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Негізгі капиталға тартылған инвестиция 5,5 триллион теңгені құрады</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>fake_number</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Негізгі капиталға тартылған инвестиция көлемі 9,5 триллион теңгені құрады</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
       <c r="J24" s="4" t="n"/>
@@ -2092,13 +2177,41 @@
       <c r="AB24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="n"/>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>024</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Биыл өңдеу секторында 1,7 триллион теңгеге 200 инвестициялық жоба іске қосылып, 17 мың жұмыс орны ашылады. Үкімет басшысы ірі автожол жобаларының жүзеге асырылу барысы, Астана қаласындағы екінші әуежайдың құрылысын және Tarlan Astana көлік жүйесінің келесі кезеңін жоспарлау туралы айтты.</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Осы жылы 200 инвестициялық жоба жүзеге асырылады</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="4" t="n"/>
@@ -2120,13 +2233,41 @@
       <c r="AB25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="n"/>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>025</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Бектеновтың айтуы бойынша Астанада үшінші теміржол вокзалы салынатын болады</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>fake_invented</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="4" t="n"/>
       <c r="J26" s="4" t="n"/>
@@ -2148,13 +2289,41 @@
       <c r="AB26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="n"/>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>026</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Биыл өңдеу секторында 1,7 триллион теңгеге 200 инвестициялық жоба іске қосылып, 17 мың жұмыс орны ашылады. Үкімет басшысы ірі автожол жобаларының жүзеге асырылу барысы, Астана қаласындағы екінші әуежайдың құрылысын және Tarlan Astana көлік жүйесінің келесі кезеңін жоспарлау туралы айтты.</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Астанада 2-ші әуежайды салу көзделуде</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
       <c r="J27" s="4" t="n"/>
@@ -2176,13 +2345,41 @@
       <c r="AB27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="n"/>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>027</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Пайдалануға берілетін тұрғын үй көлемі 20 миллион шаршы метрге жетпек. Ауыл шаруашылығындағы өндіріс көрсеткіші 15 триллион теңгені құрап, егістік алқаптары 23,8 миллион гектарға дейін ұлғайды.</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Пайдалануға берілетін тұрғын үй көлемі 20 миллион квадрат метрге жетпек</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
       <c r="J28" s="4" t="n"/>
@@ -2204,13 +2401,41 @@
       <c r="AB28" s="4" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="n"/>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Шаруаларды қолдауға 1 триллион теңге бөлінді. Бұл ретте бюджеттің әр теңгесі 6,5 теңге жеке инвестиция тартуға септігін тигізді.</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Бюджеттен шаруаларға бөлінген 6,5 теңгесі бір теңге жеке инвестиция тартуға септігін тигізді.</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>fake_causal</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Бұл ретте бюджеттің әр теңгесі 6,5 теңге жеке инвестиция тартуға септігін тигізді.</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="4" t="n"/>
       <c r="J29" s="4" t="n"/>
@@ -2232,13 +2457,41 @@
       <c r="AB29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="n"/>
-      <c r="B30" s="4" t="n"/>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="n"/>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>029</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Мемлекет басшысына Халықтың табысын арттыру жөніндегі кешенді жоспардың іске асырылуы және инфляцияны төмендету шаралары туралы ақпарат берілді. Маусым айында жылдық инфляция деңгейі 10,3 пайызды құрады.</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Маусым айында жылдық инфляция 10,3 процент болды.</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="4" t="n"/>
       <c r="J30" s="4" t="n"/>
@@ -2260,13 +2513,41 @@
       <c r="AB30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n"/>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>030</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Президентке әлеуметтік және көші-қон саясатын жетілдіру нәтижелері туралы баяндалды, сондай-ақ жұмысқа орналасуға ынталандыру арқылы әлеуметтік қолдау тетіктерінің тиімділігін арттыру тәсілдері таныстырылды. Кейбір әлеуметтік төлемдерді оңтайландыру нәтижесінде жылына 800 миллиард теңгеден аса қаржы үнемделеді.</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Кейбір әлеуметтік төлемдерді азайту нәтижесінде жылына 801 миллиард теңгеден аса қаржы үнемделеді.</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>fake_number</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Кейбір әлеуметтік төлемдерді оңтайландыру нәтижесінде жылына 800 миллиард теңгеден аса қаржы үнемделеді.</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="4" t="n"/>
       <c r="J31" s="4" t="n"/>
@@ -2288,13 +2569,41 @@
       <c r="AB31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="n"/>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>031</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Олжас Бектенов «Деректерді өңдеу орталығы алқабы» жобасын іске асыру мақсатында әлемдік ІТ көшбасшыларымен бірге қуаты 250 МВт болатын инфрақұрылым жасақталатынын айтты.</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Қуаты 250 МВт болатын инфрақұрылымды жасақтау үшін «Деректерді өңдеу орталығы алқабы» жобасы іске қосылады.</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>fake_causal</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Олжас Бектенов «Деректерді өңдеу орталығы алқабы» жобасын іске асыру мақсатында әлемдік ІТ көшбасшыларымен бірге қуаты 250 МВт болатын инфрақұрылым жасақталатынын айтты.</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="4" t="n"/>
       <c r="J32" s="4" t="n"/>
@@ -2316,13 +2625,41 @@
       <c r="AB32" s="4" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n"/>
-      <c r="B33" s="4" t="n"/>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4" t="n"/>
-      <c r="E33" s="4" t="n"/>
-      <c r="F33" s="4" t="n"/>
-      <c r="G33" s="4" t="n"/>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>032</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Кездесуде жылыту маусымына дайындық мәселесіне айрықша назар аударылды. Өткен маусымның қорытындысы бойынша бес жылу электр орталығы аса жоғары тәуекелдің «қызыл» аймағынан шығарылып, үш ЖЭО «жасыл» аймаққа ауыстырылды. Биылғы жөндеу жұмыстары 9 энергия блогын, 55 қазандықты және 51 турбинаны қамтиды. Аталған мақсатқа 384 миллиард теңге бөлінген. «Энергетикалық және коммуналдық секторларды жаңғырту» ұлттық жобасы аясында жыл соңына дейін 12 мың шақырым инженерлік желі жөнделеді.</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Бес жылу электр орталығы тәуекелдің «қызыл» аймағынан шығарылып, үш ЖЭО «жасыл» аймаққа өтетін болады</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="4" t="n"/>
       <c r="J33" s="4" t="n"/>
@@ -2344,13 +2681,41 @@
       <c r="AB33" s="4" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="n"/>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="4" t="n"/>
-      <c r="F34" s="4" t="n"/>
-      <c r="G34" s="4" t="n"/>
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>033</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Алматы тау кластерін дамыту туризм саласының ІЖӨ құрылымындағы үлесін арттырады.</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Туризм саласының ІЖӨ құрылымындағы үлесінің артуы Алматы тау кластерін дамытуды шапшаңдатады.</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>fake_causal</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Алматы тау кластерін дамыту туризм саласының ІЖӨ құрылымындағы үлесін арттырады.</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H34" s="4" t="n"/>
       <c r="I34" s="4" t="n"/>
       <c r="J34" s="4" t="n"/>
@@ -2372,13 +2737,41 @@
       <c r="AB34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="n"/>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="4" t="n"/>
-      <c r="G35" s="4" t="n"/>
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>034</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Президент халық коньки тебетін "Медеу" алқабын қайта құруға қаражат бөлуге тапсырма берді.</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>fake_invented</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
       <c r="J35" s="4" t="n"/>
@@ -2400,13 +2793,41 @@
       <c r="AB35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n"/>
-      <c r="B36" s="4" t="n"/>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="4" t="n"/>
-      <c r="G36" s="4" t="n"/>
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>035</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Almaty SuperSki жобасының құрылысы жандана түсті: 60 шақырым трасса құрылысы аяқталғанда тәулігіне 10 мың адамға дейін қызмет көрсетуге мүмкіндік туады. </t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Almaty SuperSki жобасы бойынша тәулігіне 10 мың адам қызмет алса, 60 шағырым трасса аяқталатын болады.</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>fake_causal</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>60 шақырым трасса құрылысы аяқталғанда тәулігіне 10 мың адамға дейін қызмет көрсетуге мүмкіндік туады</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="4" t="n"/>
       <c r="J36" s="4" t="n"/>
@@ -2428,13 +2849,41 @@
       <c r="AB36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="n"/>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>036</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Бектенов Тоқаевқа жаңа стадион салу туралы ұсыныс жасады.</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>fake_invented</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
       <c r="J37" s="4" t="n"/>
@@ -2456,13 +2905,41 @@
       <c r="AB37" s="4" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="n"/>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>037</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Нысанды пайдалануға беру 2028 жылдың желтоқсан айына жоспарланған. Еліміз «Болашақ ойындары-2026» жарыстарын өткізуге дайын.</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Қазақстан «Ескі Қазақстан ойындары-2026» жарыстарын өткізуге дайын.</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>fake_entity</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Еліміз «Болашақ ойындары-2026» жарыстарын өткізуге дайын.</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="4" t="n"/>
       <c r="J38" s="4" t="n"/>
@@ -2484,13 +2961,41 @@
       <c r="AB38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="n"/>
-      <c r="B39" s="4" t="n"/>
-      <c r="C39" s="4" t="n"/>
-      <c r="D39" s="4" t="n"/>
-      <c r="E39" s="4" t="n"/>
-      <c r="F39" s="4" t="n"/>
-      <c r="G39" s="4" t="n"/>
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>038</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Биылғы жөндеу жұмыстары 9 энергия блогын, 55 қазандықты және 51 турбинаны қамтиды. Аталған мақсатқа 384 миллиард теңге бөлінген.</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Осы жылғы жөндеу жұмыстары 11 энергия блогын қамтиды.</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>fake_number</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Биылғы жөндеу жұмыстары 9 энергия блогын, 55 қазандықты және 51 турбинаны қамтиды. </t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="4" t="n"/>
       <c r="J39" s="4" t="n"/>
@@ -2512,13 +3017,41 @@
       <c r="AB39" s="4" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="n"/>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="n"/>
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>039</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Кездесу соңында Президент пен Премьер-Министр фотосуретке түсті.</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>fake_invented</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="4" t="n"/>
       <c r="J40" s="4" t="n"/>
@@ -2540,13 +3073,41 @@
       <c r="AB40" s="4" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="n"/>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="4" t="n"/>
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>040</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Мемлекет басшысы жаңа Конституцияға сай қабылданып жатқан шаралар туралы хабардар болды. Заңнаманы Ата заңға сәйкестендіру, «Әділетті Қазақстан» және «Заң мен тәртіп» қағидаттарын нығайту, әлеуметтік саясатты жетілдіру, Алатау қаласын қарқынды дамыту үшін құқықтық негіз қалыптастыру, сондай-ақ «Таза Қазақстан» бастамасын ілгерілету бойынша жұмыстар жүргізілуде.</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Бектенов Президентке жаңа Конституцияға байланысты қабылданып жатқан іс-әрекеттер туралы баяндады.</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="H41" s="4" t="n"/>
       <c r="I41" s="4" t="n"/>
       <c r="J41" s="4" t="n"/>
@@ -2568,13 +3129,41 @@
       <c r="AB41" s="4" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="n"/>
-      <c r="B42" s="4" t="n"/>
-      <c r="C42" s="4" t="n"/>
-      <c r="D42" s="4" t="n"/>
-      <c r="E42" s="4" t="n"/>
-      <c r="F42" s="4" t="n"/>
-      <c r="G42" s="4" t="n"/>
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>041</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>news_text1</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Кездесу барысында Бектенов ауырып жатқанын айтып, Тоқаевтан еңбек демалысына жіберуді өтінді</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>fake_invented</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="H42" s="4" t="n"/>
       <c r="I42" s="4" t="n"/>
       <c r="J42" s="4" t="n"/>

</xml_diff>

<commit_message>
Add Claude blind run on news_text1 (20/21, 100% grounded)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -2047,7 +2047,11 @@
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="4" t="n"/>
       <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="n"/>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N22" s="4" t="n"/>
       <c r="O22" s="4" t="n"/>
       <c r="P22" s="4" t="n"/>
@@ -2103,7 +2107,11 @@
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
       <c r="J23" s="4" t="n"/>
-      <c r="K23" s="4" t="n"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N23" s="4" t="n"/>
       <c r="O23" s="4" t="n"/>
       <c r="P23" s="4" t="n"/>
@@ -2159,7 +2167,11 @@
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
       <c r="J24" s="4" t="n"/>
-      <c r="K24" s="4" t="n"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N24" s="4" t="n"/>
       <c r="O24" s="4" t="n"/>
       <c r="P24" s="4" t="n"/>
@@ -2215,7 +2227,11 @@
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="4" t="n"/>
-      <c r="K25" s="4" t="n"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N25" s="4" t="n"/>
       <c r="O25" s="4" t="n"/>
       <c r="P25" s="4" t="n"/>
@@ -2271,7 +2287,11 @@
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="4" t="n"/>
       <c r="J26" s="4" t="n"/>
-      <c r="K26" s="4" t="n"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="N26" s="4" t="n"/>
       <c r="O26" s="4" t="n"/>
       <c r="P26" s="4" t="n"/>
@@ -2327,7 +2347,11 @@
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
       <c r="J27" s="4" t="n"/>
-      <c r="K27" s="4" t="n"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N27" s="4" t="n"/>
       <c r="O27" s="4" t="n"/>
       <c r="P27" s="4" t="n"/>
@@ -2383,7 +2407,11 @@
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
       <c r="J28" s="4" t="n"/>
-      <c r="K28" s="4" t="n"/>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N28" s="4" t="n"/>
       <c r="O28" s="4" t="n"/>
       <c r="P28" s="4" t="n"/>
@@ -2439,7 +2467,11 @@
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="4" t="n"/>
       <c r="J29" s="4" t="n"/>
-      <c r="K29" s="4" t="n"/>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N29" s="4" t="n"/>
       <c r="O29" s="4" t="n"/>
       <c r="P29" s="4" t="n"/>
@@ -2495,7 +2527,11 @@
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="4" t="n"/>
       <c r="J30" s="4" t="n"/>
-      <c r="K30" s="4" t="n"/>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N30" s="4" t="n"/>
       <c r="O30" s="4" t="n"/>
       <c r="P30" s="4" t="n"/>
@@ -2551,7 +2587,11 @@
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="4" t="n"/>
       <c r="J31" s="4" t="n"/>
-      <c r="K31" s="4" t="n"/>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N31" s="4" t="n"/>
       <c r="O31" s="4" t="n"/>
       <c r="P31" s="4" t="n"/>
@@ -2607,7 +2647,11 @@
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="4" t="n"/>
       <c r="J32" s="4" t="n"/>
-      <c r="K32" s="4" t="n"/>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N32" s="4" t="n"/>
       <c r="O32" s="4" t="n"/>
       <c r="P32" s="4" t="n"/>
@@ -2663,7 +2707,11 @@
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="4" t="n"/>
       <c r="J33" s="4" t="n"/>
-      <c r="K33" s="4" t="n"/>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N33" s="4" t="n"/>
       <c r="O33" s="4" t="n"/>
       <c r="P33" s="4" t="n"/>
@@ -2719,7 +2767,11 @@
       <c r="H34" s="4" t="n"/>
       <c r="I34" s="4" t="n"/>
       <c r="J34" s="4" t="n"/>
-      <c r="K34" s="4" t="n"/>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N34" s="4" t="n"/>
       <c r="O34" s="4" t="n"/>
       <c r="P34" s="4" t="n"/>
@@ -2775,7 +2827,11 @@
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
       <c r="J35" s="4" t="n"/>
-      <c r="K35" s="4" t="n"/>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="N35" s="4" t="n"/>
       <c r="O35" s="4" t="n"/>
       <c r="P35" s="4" t="n"/>
@@ -2831,7 +2887,11 @@
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="4" t="n"/>
       <c r="J36" s="4" t="n"/>
-      <c r="K36" s="4" t="n"/>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N36" s="4" t="n"/>
       <c r="O36" s="4" t="n"/>
       <c r="P36" s="4" t="n"/>
@@ -2887,7 +2947,11 @@
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
       <c r="J37" s="4" t="n"/>
-      <c r="K37" s="4" t="n"/>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="N37" s="4" t="n"/>
       <c r="O37" s="4" t="n"/>
       <c r="P37" s="4" t="n"/>
@@ -2943,7 +3007,11 @@
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="4" t="n"/>
       <c r="J38" s="4" t="n"/>
-      <c r="K38" s="4" t="n"/>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N38" s="4" t="n"/>
       <c r="O38" s="4" t="n"/>
       <c r="P38" s="4" t="n"/>
@@ -2999,7 +3067,11 @@
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="4" t="n"/>
       <c r="J39" s="4" t="n"/>
-      <c r="K39" s="4" t="n"/>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N39" s="4" t="n"/>
       <c r="O39" s="4" t="n"/>
       <c r="P39" s="4" t="n"/>
@@ -3055,7 +3127,11 @@
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="4" t="n"/>
       <c r="J40" s="4" t="n"/>
-      <c r="K40" s="4" t="n"/>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="N40" s="4" t="n"/>
       <c r="O40" s="4" t="n"/>
       <c r="P40" s="4" t="n"/>
@@ -3111,7 +3187,11 @@
       <c r="H41" s="4" t="n"/>
       <c r="I41" s="4" t="n"/>
       <c r="J41" s="4" t="n"/>
-      <c r="K41" s="4" t="n"/>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N41" s="4" t="n"/>
       <c r="O41" s="4" t="n"/>
       <c r="P41" s="4" t="n"/>
@@ -3167,7 +3247,11 @@
       <c r="H42" s="4" t="n"/>
       <c r="I42" s="4" t="n"/>
       <c r="J42" s="4" t="n"/>
-      <c r="K42" s="4" t="n"/>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="N42" s="4" t="n"/>
       <c r="O42" s="4" t="n"/>
       <c r="P42" s="4" t="n"/>

</xml_diff>

<commit_message>
Refine claim 021: month-only date change (13 шілде->13 маусым), type fake_number
- 022 kept as fake_entity (fact negation, contradicts source) per author decision
- regenerated news chat prompt with corrected 021

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -2026,17 +2026,17 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Тоқаев Бектеновпен 2 маусымда кездесті.</t>
+          <t>Тоқаев Бектеновпен 13 маусымда кездесті.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>fake_entity</t>
+          <t>fake_number</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026 жылғы 13 шілдеде мемлекет басшысы Премьер-министр Олжас Бектеновті қабылдады. </t>
+          <t>«13 шілдеде» → «13 маусымда» (ай ауыстырылды)</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">

</xml_diff>

<commit_message>
DeepSeek news_text1 run (19/21); make grounding check case-insensitive
- check_grounding.py casefolds so a capitalised first letter of a mid-sentence
  quote is not falsely flagged (DeepSeek 022/028 were false negatives -> now 100%)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -2046,7 +2046,11 @@
       </c>
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="4" t="n"/>
-      <c r="J22" s="4" t="n"/>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -2106,7 +2110,11 @@
       </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
-      <c r="J23" s="4" t="n"/>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -2166,7 +2174,11 @@
       </c>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
-      <c r="J24" s="4" t="n"/>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -2226,7 +2238,11 @@
       </c>
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
-      <c r="J25" s="4" t="n"/>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -2286,7 +2302,11 @@
       </c>
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="4" t="n"/>
-      <c r="J26" s="4" t="n"/>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -2346,7 +2366,11 @@
       </c>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
-      <c r="J27" s="4" t="n"/>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -2406,7 +2430,11 @@
       </c>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
-      <c r="J28" s="4" t="n"/>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -2466,7 +2494,11 @@
       </c>
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="4" t="n"/>
-      <c r="J29" s="4" t="n"/>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -2526,7 +2558,11 @@
       </c>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="4" t="n"/>
-      <c r="J30" s="4" t="n"/>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -2586,7 +2622,11 @@
       </c>
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="4" t="n"/>
-      <c r="J31" s="4" t="n"/>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -2646,7 +2686,11 @@
       </c>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="4" t="n"/>
-      <c r="J32" s="4" t="n"/>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -2706,7 +2750,11 @@
       </c>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="4" t="n"/>
-      <c r="J33" s="4" t="n"/>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -2766,7 +2814,11 @@
       </c>
       <c r="H34" s="4" t="n"/>
       <c r="I34" s="4" t="n"/>
-      <c r="J34" s="4" t="n"/>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -2826,7 +2878,11 @@
       </c>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
-      <c r="J35" s="4" t="n"/>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -2886,7 +2942,11 @@
       </c>
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="4" t="n"/>
-      <c r="J36" s="4" t="n"/>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -2946,7 +3006,11 @@
       </c>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
-      <c r="J37" s="4" t="n"/>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -3006,7 +3070,11 @@
       </c>
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="4" t="n"/>
-      <c r="J38" s="4" t="n"/>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -3066,7 +3134,11 @@
       </c>
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="4" t="n"/>
-      <c r="J39" s="4" t="n"/>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -3126,7 +3198,11 @@
       </c>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="4" t="n"/>
-      <c r="J40" s="4" t="n"/>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -3186,7 +3262,11 @@
       </c>
       <c r="H41" s="4" t="n"/>
       <c r="I41" s="4" t="n"/>
-      <c r="J41" s="4" t="n"/>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -3246,7 +3326,11 @@
       </c>
       <c r="H42" s="4" t="n"/>
       <c r="I42" s="4" t="n"/>
-      <c r="J42" s="4" t="n"/>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>

</xml_diff>

<commit_message>
Qwen news_text1 run (18/21, 100% grounded)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -2056,6 +2056,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N22" s="4" t="n"/>
       <c r="O22" s="4" t="n"/>
       <c r="P22" s="4" t="n"/>
@@ -2120,6 +2125,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N23" s="4" t="n"/>
       <c r="O23" s="4" t="n"/>
       <c r="P23" s="4" t="n"/>
@@ -2184,6 +2194,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N24" s="4" t="n"/>
       <c r="O24" s="4" t="n"/>
       <c r="P24" s="4" t="n"/>
@@ -2248,6 +2263,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N25" s="4" t="n"/>
       <c r="O25" s="4" t="n"/>
       <c r="P25" s="4" t="n"/>
@@ -2312,6 +2332,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N26" s="4" t="n"/>
       <c r="O26" s="4" t="n"/>
       <c r="P26" s="4" t="n"/>
@@ -2376,6 +2401,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N27" s="4" t="n"/>
       <c r="O27" s="4" t="n"/>
       <c r="P27" s="4" t="n"/>
@@ -2440,6 +2470,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N28" s="4" t="n"/>
       <c r="O28" s="4" t="n"/>
       <c r="P28" s="4" t="n"/>
@@ -2504,6 +2539,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N29" s="4" t="n"/>
       <c r="O29" s="4" t="n"/>
       <c r="P29" s="4" t="n"/>
@@ -2568,6 +2608,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N30" s="4" t="n"/>
       <c r="O30" s="4" t="n"/>
       <c r="P30" s="4" t="n"/>
@@ -2632,6 +2677,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N31" s="4" t="n"/>
       <c r="O31" s="4" t="n"/>
       <c r="P31" s="4" t="n"/>
@@ -2696,6 +2746,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N32" s="4" t="n"/>
       <c r="O32" s="4" t="n"/>
       <c r="P32" s="4" t="n"/>
@@ -2760,6 +2815,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N33" s="4" t="n"/>
       <c r="O33" s="4" t="n"/>
       <c r="P33" s="4" t="n"/>
@@ -2824,6 +2884,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N34" s="4" t="n"/>
       <c r="O34" s="4" t="n"/>
       <c r="P34" s="4" t="n"/>
@@ -2888,6 +2953,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="N35" s="4" t="n"/>
       <c r="O35" s="4" t="n"/>
       <c r="P35" s="4" t="n"/>
@@ -2952,6 +3022,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N36" s="4" t="n"/>
       <c r="O36" s="4" t="n"/>
       <c r="P36" s="4" t="n"/>
@@ -3016,6 +3091,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="N37" s="4" t="n"/>
       <c r="O37" s="4" t="n"/>
       <c r="P37" s="4" t="n"/>
@@ -3080,6 +3160,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N38" s="4" t="n"/>
       <c r="O38" s="4" t="n"/>
       <c r="P38" s="4" t="n"/>
@@ -3144,6 +3229,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="N39" s="4" t="n"/>
       <c r="O39" s="4" t="n"/>
       <c r="P39" s="4" t="n"/>
@@ -3208,6 +3298,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="N40" s="4" t="n"/>
       <c r="O40" s="4" t="n"/>
       <c r="P40" s="4" t="n"/>
@@ -3272,6 +3367,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="N41" s="4" t="n"/>
       <c r="O41" s="4" t="n"/>
       <c r="P41" s="4" t="n"/>
@@ -3332,6 +3432,11 @@
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>

</xml_diff>

<commit_message>
Kimi news_text1 run (20/21, 100% grounded)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -2056,7 +2056,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="M22" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2125,7 +2130,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="M23" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2194,7 +2204,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="M24" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2263,7 +2278,12 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
+      <c r="M25" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -2332,7 +2352,12 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
+      <c r="M26" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2401,7 +2426,12 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
+      <c r="M27" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -2470,7 +2500,12 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
+      <c r="M28" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -2539,7 +2574,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="M29" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2608,7 +2648,12 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
+      <c r="M30" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -2677,7 +2722,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="M31" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2746,7 +2796,12 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="M32" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -2815,7 +2870,12 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="M33" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2884,7 +2944,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="M34" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2953,7 +3018,12 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
+      <c r="M35" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -3022,7 +3092,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="M36" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -3091,7 +3166,12 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
+      <c r="M37" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -3160,7 +3240,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="M38" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -3229,7 +3314,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="M39" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -3298,7 +3388,12 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
+      <c r="M40" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -3367,7 +3462,12 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
+      <c r="M41" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -3436,7 +3536,12 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
+      <c r="M42" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>

</xml_diff>

<commit_message>
Complete text 2 (all 5 models); add leaderboard.py
- Gemini news_text1 run (19/21); unify Claude model field for aggregation
- scripts/leaderboard.py: combined per-model scoring across sources with
  Wilson CIs, macro-F1, per-type and per-source breakdowns

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -2044,7 +2044,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H22" s="4" t="n"/>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I22" s="4" t="n"/>
       <c r="J22" s="4" t="inlineStr">
         <is>
@@ -2056,7 +2060,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="L22" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2118,7 +2122,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H23" s="4" t="n"/>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I23" s="4" t="n"/>
       <c r="J23" s="4" t="inlineStr">
         <is>
@@ -2130,7 +2138,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L23" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2192,7 +2200,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H24" s="4" t="n"/>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I24" s="4" t="n"/>
       <c r="J24" s="4" t="inlineStr">
         <is>
@@ -2204,7 +2216,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L24" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2266,7 +2278,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H25" s="4" t="n"/>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="4" t="inlineStr">
         <is>
@@ -2278,7 +2294,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="L25" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -2340,7 +2356,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="H26" s="4" t="n"/>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I26" s="4" t="n"/>
       <c r="J26" s="4" t="inlineStr">
         <is>
@@ -2352,7 +2372,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L26" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -2414,7 +2434,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H27" s="4" t="n"/>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I27" s="4" t="n"/>
       <c r="J27" s="4" t="inlineStr">
         <is>
@@ -2426,7 +2450,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L27" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -2488,7 +2512,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H28" s="4" t="n"/>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I28" s="4" t="n"/>
       <c r="J28" s="4" t="inlineStr">
         <is>
@@ -2500,7 +2528,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L28" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -2562,7 +2590,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H29" s="4" t="n"/>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I29" s="4" t="n"/>
       <c r="J29" s="4" t="inlineStr">
         <is>
@@ -2574,7 +2606,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L29" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2636,7 +2668,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H30" s="4" t="n"/>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I30" s="4" t="n"/>
       <c r="J30" s="4" t="inlineStr">
         <is>
@@ -2648,7 +2684,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="L30" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -2710,7 +2746,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H31" s="4" t="n"/>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I31" s="4" t="n"/>
       <c r="J31" s="4" t="inlineStr">
         <is>
@@ -2722,7 +2762,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="L31" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2784,7 +2824,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H32" s="4" t="n"/>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I32" s="4" t="n"/>
       <c r="J32" s="4" t="inlineStr">
         <is>
@@ -2796,7 +2840,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L32" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2858,7 +2902,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H33" s="4" t="n"/>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I33" s="4" t="n"/>
       <c r="J33" s="4" t="inlineStr">
         <is>
@@ -2870,7 +2918,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="L33" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -2932,7 +2980,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H34" s="4" t="n"/>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I34" s="4" t="n"/>
       <c r="J34" s="4" t="inlineStr">
         <is>
@@ -2944,7 +2996,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L34" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -3006,7 +3058,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="H35" s="4" t="n"/>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I35" s="4" t="n"/>
       <c r="J35" s="4" t="inlineStr">
         <is>
@@ -3018,7 +3074,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="L35" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -3080,7 +3136,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H36" s="4" t="n"/>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I36" s="4" t="n"/>
       <c r="J36" s="4" t="inlineStr">
         <is>
@@ -3092,7 +3152,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="L36" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -3154,7 +3214,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="H37" s="4" t="n"/>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I37" s="4" t="n"/>
       <c r="J37" s="4" t="inlineStr">
         <is>
@@ -3166,7 +3230,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="L37" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -3228,7 +3292,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H38" s="4" t="n"/>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I38" s="4" t="n"/>
       <c r="J38" s="4" t="inlineStr">
         <is>
@@ -3240,7 +3308,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="L38" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -3302,7 +3370,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H39" s="4" t="n"/>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I39" s="4" t="n"/>
       <c r="J39" s="4" t="inlineStr">
         <is>
@@ -3314,7 +3386,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="L39" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -3376,7 +3448,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="H40" s="4" t="n"/>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I40" s="4" t="n"/>
       <c r="J40" s="4" t="inlineStr">
         <is>
@@ -3388,7 +3464,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="L40" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -3450,7 +3526,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H41" s="4" t="n"/>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I41" s="4" t="n"/>
       <c r="J41" s="4" t="inlineStr">
         <is>
@@ -3462,7 +3542,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L41" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -3524,7 +3604,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="H42" s="4" t="n"/>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I42" s="4" t="n"/>
       <c r="J42" s="4" t="inlineStr">
         <is>
@@ -3536,7 +3620,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L42" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>

</xml_diff>

<commit_message>
Correct claim 032 (tense artifact); re-evaluate affected models
- claim 032 was a 'real' item with an unintended future-tense phrasing
  (өтетін болады) vs the source's past tense; changed to өтті
- Qwen and Kimi had marked it REFUTED solely on that tense difference (per
  their rationale); post-hoc corrected to SUPPORTED with original verdict and
  a correction_note preserved in the result files for audit
- Claude/Gemini/DeepSeek already answered SUPPORTED (unaffected)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -2884,7 +2884,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Бес жылу электр орталығы тәуекелдің «қызыл» аймағынан шығарылып, үш ЖЭО «жасыл» аймаққа өтетін болады</t>
+          <t>Бес жылу электр орталығы тәуекелдің «қызыл» аймағынан шығарылып, үш ЖЭО «жасыл» аймаққа өтті</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -2920,12 +2920,12 @@
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t>REFUTED</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="M33" s="0" t="inlineStr">
         <is>
-          <t>REFUTED</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="N33" s="4" t="n"/>

</xml_diff>

<commit_message>
Integrate text 3 (msgtxt): 19 claims (042-060), 60 total
- fake_invented items 045/051/053/059 labeled NOT_ENOUGH_INFO (per convention);
  052 kept fake_causal/REFUTED
- generated prompts/chat_run_msgtxt.txt

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -3601,13 +3601,42 @@
       <c r="AA42" s="4" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="n"/>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="4" t="n"/>
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>042</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Астанадан прямой рейс бар екен Эйр Астанамен. Жазира тапты билеттерді, кеше скидкамен сатып тастадық.
+</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Бека мен Жазираның отбасымен Камраньға тікелей рейспен ұшады.</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="H43" s="4" t="n"/>
       <c r="I43" s="4" t="n"/>
       <c r="J43" s="4" t="n"/>
@@ -3628,13 +3657,42 @@
       <c r="AA43" s="4" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="n"/>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
-      <c r="E44" s="4" t="n"/>
-      <c r="F44" s="4" t="n"/>
-      <c r="G44" s="4" t="n"/>
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>043</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ал мен 20 қыркүйекте Алматыға барам, там Медеуде концерт болады, соған вип билет алдым.
+</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Азамат 20 қыркүйекте Медеуде өтетін концертке барады.</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="H44" s="4" t="n"/>
       <c r="I44" s="4" t="n"/>
       <c r="J44" s="4" t="n"/>
@@ -3655,13 +3713,42 @@
       <c r="AA44" s="4" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="n"/>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="4" t="n"/>
-      <c r="D45" s="4" t="n"/>
-      <c r="E45" s="4" t="n"/>
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="4" t="n"/>
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>044</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Біздің толпа ғой. Төрт взрослый, үш бала. Соған қазір гостиница брондап, бас қатыватыр. Сол жаққа барып, бассейнге түсем рахаттанып.
+</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Вьетнамға ұшатын топтың ішінде бес бала бар.</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>fake_number</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>3 бала 5-ке ауыстырылды.</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H45" s="4" t="n"/>
       <c r="I45" s="4" t="n"/>
       <c r="J45" s="4" t="n"/>
@@ -3682,13 +3769,41 @@
       <c r="AA45" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="n"/>
-      <c r="B46" s="4" t="n"/>
-      <c r="C46" s="4" t="n"/>
-      <c r="D46" s="4" t="n"/>
-      <c r="E46" s="4" t="n"/>
-      <c r="F46" s="4" t="n"/>
-      <c r="G46" s="4" t="n"/>
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>045</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Азамат концерттен кейін достарымен Медеуде сырғанақ тебуді жоспарлап отыр.</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>fake_invented</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="H46" s="4" t="n"/>
       <c r="I46" s="4" t="n"/>
       <c r="J46" s="4" t="n"/>
@@ -3709,13 +3824,42 @@
       <c r="AA46" s="4" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="n"/>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
-      <c r="F47" s="4" t="n"/>
-      <c r="G47" s="4" t="n"/>
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>046</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Скриптонит қой, полный живой звук болады деді. Прикинь в ате толпа фанатов наверное будет, бакад аман болсын.
+</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Азамат Алматыға Jah Khalib-тің концертіне барады.</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>fake_entity</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Скриптонит Jah Khalib-ке ауыстырылды.</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H47" s="4" t="n"/>
       <c r="I47" s="4" t="n"/>
       <c r="J47" s="4" t="n"/>
@@ -3736,13 +3880,42 @@
       <c r="AA47" s="4" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="n"/>
-      <c r="B48" s="4" t="n"/>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="4" t="n"/>
-      <c r="E48" s="4" t="n"/>
-      <c r="F48" s="4" t="n"/>
-      <c r="G48" s="4" t="n"/>
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>047</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Жоқ, прикинь, Астанадан прямой рейс бар екен Эйр Астанамен. Жазира тапты билеттерді, кеше скидкамен сатып алдық.
+</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Камраньға ұшатын билеттерді Бека өзі тауып сатып алған.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>fake_entity</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Жазира Бекаға ауыстырылды.</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H48" s="4" t="n"/>
       <c r="I48" s="4" t="n"/>
       <c r="J48" s="4" t="n"/>
@@ -3763,13 +3936,42 @@
       <c r="AA48" s="4" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="4" t="n"/>
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>048</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Біздің толпа ғой. Төрт взрослый, үш бала. Соған қазір гостиница брондап, бас қатыватыр.
+</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Вьетнамға баратын топта төрт ересек және үш бала бар.</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="H49" s="4" t="n"/>
       <c r="I49" s="4" t="n"/>
       <c r="J49" s="4" t="n"/>
@@ -3790,13 +3992,42 @@
       <c r="AA49" s="4" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="n"/>
-      <c r="B50" s="4" t="n"/>
-      <c r="C50" s="4" t="n"/>
-      <c r="D50" s="4" t="n"/>
-      <c r="E50" s="4" t="n"/>
-      <c r="F50" s="4" t="n"/>
-      <c r="G50" s="4" t="n"/>
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>049</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Астанадан прямой рейс бар екен Эйр Астанамен. Жазира тапты билеттерді, кеше скидкамен сатып тастадық.
+</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Билеттерді Жазира жеңілдікпен сатып алды.</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="H50" s="4" t="n"/>
       <c r="I50" s="4" t="n"/>
       <c r="J50" s="4" t="n"/>
@@ -3817,13 +4048,42 @@
       <c r="AA50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="n"/>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="4" t="n"/>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="4" t="n"/>
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>050</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Короче, біз 12 тамызда Камраньға ұшатын болдық. Вьетнамға.
+</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Бека отбасымен Вьетнамға 15 тамызда ұшатын болды.</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>fake_number</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>12 саны 15-ке (күн) ауыстырылды.</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H51" s="4" t="n"/>
       <c r="I51" s="4" t="n"/>
       <c r="J51" s="4" t="n"/>
@@ -3844,13 +4104,41 @@
       <c r="AA51" s="4" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="n"/>
-      <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="4" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
-      <c r="G52" s="4" t="n"/>
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>051</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Беканың отбасы Вьетнамда бес жұлдызды "Rixos" қонақүйінде тоқтайды.</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>fake_invented</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="H52" s="4" t="n"/>
       <c r="I52" s="4" t="n"/>
       <c r="J52" s="4" t="n"/>
@@ -3871,13 +4159,43 @@
       <c r="AA52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="n"/>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
-      <c r="E53" s="4" t="n"/>
-      <c r="F53" s="4" t="n"/>
-      <c r="G53" s="4" t="n"/>
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>052</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Скриптонит қой, полный живой звук болады деді. Прикинь в ате толпа фанатов наверное будет, бакад аман болсын.
+</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Алматыда кептелістер салдарынан Скриптониттің концерті өтетін болады</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>fake_causal</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Скриптонит қой, полный живой звук болады деді. Прикинь в ате толпа фанатов наверное будет, бакад аман болсын.
+</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H53" s="4" t="n"/>
       <c r="I53" s="4" t="n"/>
       <c r="J53" s="4" t="n"/>
@@ -3898,13 +4216,41 @@
       <c r="AA53" s="4" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="n"/>
-      <c r="B54" s="4" t="n"/>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="4" t="n"/>
-      <c r="E54" s="4" t="n"/>
-      <c r="F54" s="4" t="n"/>
-      <c r="G54" s="4" t="n"/>
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>053</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Азамат транзитпен айналысатын компанияда қызмет етеді</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>fake_invented</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="H54" s="4" t="n"/>
       <c r="I54" s="4" t="n"/>
       <c r="J54" s="4" t="n"/>
@@ -3925,13 +4271,43 @@
       <c r="AA54" s="4" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="n"/>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
-      <c r="E55" s="4" t="n"/>
-      <c r="F55" s="4" t="n"/>
-      <c r="G55" s="4" t="n"/>
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>054</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Жоқ, прикинь, Астанадан прямой рейс бар екен Эйр Астанамен. Жазира тапты билеттерді, кеше скидкамен сатып алдық.
+</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Астанадан тікелей рейспен ұшып барып, содан кейін билеттерді сатып алды.</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>fake_causal</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Жоқ, прикинь, Астанадан прямой рейс бар екен Эйр Астанамен. Жазира тапты билеттерді, кеше скидкамен сатып алдық.
+</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H55" s="4" t="n"/>
       <c r="I55" s="4" t="n"/>
       <c r="J55" s="4" t="n"/>
@@ -3952,13 +4328,41 @@
       <c r="AA55" s="4" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="n"/>
-      <c r="B56" s="4" t="n"/>
-      <c r="C56" s="4" t="n"/>
-      <c r="D56" s="4" t="n"/>
-      <c r="E56" s="4" t="n"/>
-      <c r="F56" s="4" t="n"/>
-      <c r="G56" s="4" t="n"/>
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>055</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Біздің толпа ғой. Төрт взрослый, үш бала. Соған қазір гостиница брондап, бас қатыватыр. Сол жаққа барып, бассейнге түсем рахаттанып.</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Бека бассейнге түсіп, ал кейін қонақ үйде бөлме жалдайтын болады.</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>fake_causal</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Біздің толпа ғой. Төрт взрослый, үш бала. Соған қазір гостиница брондап, бас қатыватыр. Сол жаққа барып, бассейнге түсем рахаттанып.</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H56" s="4" t="n"/>
       <c r="I56" s="4" t="n"/>
       <c r="J56" s="4" t="n"/>
@@ -3979,13 +4383,41 @@
       <c r="AA56" s="4" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="n"/>
-      <c r="B57" s="4" t="n"/>
-      <c r="C57" s="4" t="n"/>
-      <c r="D57" s="4" t="n"/>
-      <c r="E57" s="4" t="n"/>
-      <c r="F57" s="4" t="n"/>
-      <c r="G57" s="4" t="n"/>
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>056</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Біздің толпа ғой. Төрт взрослый, үш бала. Соған қазір гостиница брондап, бас қатыватыр. Сол жаққа барып, бассейнге түсем рахаттанып.</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Вьетнамға баратын топта екі ересек бар.</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>fake_number</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>4 ересек 2-ге ауыстырылды.</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H57" s="4" t="n"/>
       <c r="I57" s="4" t="n"/>
       <c r="J57" s="4" t="n"/>
@@ -4006,13 +4438,42 @@
       <c r="AA57" s="4" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="n"/>
-      <c r="B58" s="4" t="n"/>
-      <c r="C58" s="4" t="n"/>
-      <c r="D58" s="4" t="n"/>
-      <c r="E58" s="4" t="n"/>
-      <c r="F58" s="4" t="n"/>
-      <c r="G58" s="4" t="n"/>
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>057</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Короче, біз 12 тамызда Камраньға ұшатын болдық. Вьетнамға.
+</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Беканың семьясы демалысқа Түркияға ұшатын болды.</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>fake_entity</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>Вьетнам Түркияға ауыстырылды.</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H58" s="4" t="n"/>
       <c r="I58" s="4" t="n"/>
       <c r="J58" s="4" t="n"/>
@@ -4033,13 +4494,42 @@
       <c r="AA58" s="4" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="n"/>
-      <c r="B59" s="4" t="n"/>
-      <c r="C59" s="4" t="n"/>
-      <c r="D59" s="4" t="n"/>
-      <c r="E59" s="4" t="n"/>
-      <c r="F59" s="4" t="n"/>
-      <c r="G59" s="4" t="n"/>
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>058</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Керемет. Ал мен 20 қыркүйекте Алматыға барам, там Медеуде концерт болады, соған вип билет алдым.
+</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Азамат Алматыдағы концертке 10 қыркүйекте барады.</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>fake_number</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>20 саны 10-ға (күн) ауыстырылды.</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H59" s="4" t="n"/>
       <c r="I59" s="4" t="n"/>
       <c r="J59" s="4" t="n"/>
@@ -4060,13 +4550,41 @@
       <c r="AA59" s="4" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="n"/>
-      <c r="B60" s="4" t="n"/>
-      <c r="C60" s="4" t="n"/>
-      <c r="D60" s="4" t="n"/>
-      <c r="E60" s="4" t="n"/>
-      <c r="F60" s="4" t="n"/>
-      <c r="G60" s="4" t="n"/>
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>059</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Жазира Камраньға билеттерді Kaspi арқылы бөліп төлеуге алды.</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>fake_invented</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="H60" s="4" t="n"/>
       <c r="I60" s="4" t="n"/>
       <c r="J60" s="4" t="n"/>
@@ -4087,13 +4605,42 @@
       <c r="AA60" s="4" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="n"/>
-      <c r="B61" s="4" t="n"/>
-      <c r="C61" s="4" t="n"/>
-      <c r="D61" s="4" t="n"/>
-      <c r="E61" s="4" t="n"/>
-      <c r="F61" s="4" t="n"/>
-      <c r="G61" s="4" t="n"/>
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>060</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>msgtxt</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Жоқ, прикинь, Астанадан прямой рейс бар екен Эйр Астанамен. Жазира тапты билеттерді, кеше скидкамен сатып алдық.
+</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Беканың отбасы Вьетнамға Scat авиакомпаниясымен ұшады.</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>fake_entity</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Air Astana Scat-қа ауыстырылды.</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="H61" s="4" t="n"/>
       <c r="I61" s="4" t="n"/>
       <c r="J61" s="4" t="n"/>

</xml_diff>

<commit_message>
Add Claude blind run on msgtxt (19/19, 100% grounded)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -3639,7 +3639,11 @@
       </c>
       <c r="H43" s="4" t="n"/>
       <c r="I43" s="4" t="n"/>
-      <c r="J43" s="4" t="n"/>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="M43" s="4" t="n"/>
       <c r="N43" s="4" t="n"/>
       <c r="O43" s="4" t="n"/>
@@ -3695,7 +3699,11 @@
       </c>
       <c r="H44" s="4" t="n"/>
       <c r="I44" s="4" t="n"/>
-      <c r="J44" s="4" t="n"/>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="M44" s="4" t="n"/>
       <c r="N44" s="4" t="n"/>
       <c r="O44" s="4" t="n"/>
@@ -3751,7 +3759,11 @@
       </c>
       <c r="H45" s="4" t="n"/>
       <c r="I45" s="4" t="n"/>
-      <c r="J45" s="4" t="n"/>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M45" s="4" t="n"/>
       <c r="N45" s="4" t="n"/>
       <c r="O45" s="4" t="n"/>
@@ -3806,7 +3818,11 @@
       </c>
       <c r="H46" s="4" t="n"/>
       <c r="I46" s="4" t="n"/>
-      <c r="J46" s="4" t="n"/>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="M46" s="4" t="n"/>
       <c r="N46" s="4" t="n"/>
       <c r="O46" s="4" t="n"/>
@@ -3862,7 +3878,11 @@
       </c>
       <c r="H47" s="4" t="n"/>
       <c r="I47" s="4" t="n"/>
-      <c r="J47" s="4" t="n"/>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M47" s="4" t="n"/>
       <c r="N47" s="4" t="n"/>
       <c r="O47" s="4" t="n"/>
@@ -3918,7 +3938,11 @@
       </c>
       <c r="H48" s="4" t="n"/>
       <c r="I48" s="4" t="n"/>
-      <c r="J48" s="4" t="n"/>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M48" s="4" t="n"/>
       <c r="N48" s="4" t="n"/>
       <c r="O48" s="4" t="n"/>
@@ -3974,7 +3998,11 @@
       </c>
       <c r="H49" s="4" t="n"/>
       <c r="I49" s="4" t="n"/>
-      <c r="J49" s="4" t="n"/>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="M49" s="4" t="n"/>
       <c r="N49" s="4" t="n"/>
       <c r="O49" s="4" t="n"/>
@@ -4030,7 +4058,11 @@
       </c>
       <c r="H50" s="4" t="n"/>
       <c r="I50" s="4" t="n"/>
-      <c r="J50" s="4" t="n"/>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="M50" s="4" t="n"/>
       <c r="N50" s="4" t="n"/>
       <c r="O50" s="4" t="n"/>
@@ -4086,7 +4118,11 @@
       </c>
       <c r="H51" s="4" t="n"/>
       <c r="I51" s="4" t="n"/>
-      <c r="J51" s="4" t="n"/>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M51" s="4" t="n"/>
       <c r="N51" s="4" t="n"/>
       <c r="O51" s="4" t="n"/>
@@ -4141,7 +4177,11 @@
       </c>
       <c r="H52" s="4" t="n"/>
       <c r="I52" s="4" t="n"/>
-      <c r="J52" s="4" t="n"/>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="M52" s="4" t="n"/>
       <c r="N52" s="4" t="n"/>
       <c r="O52" s="4" t="n"/>
@@ -4198,7 +4238,11 @@
       </c>
       <c r="H53" s="4" t="n"/>
       <c r="I53" s="4" t="n"/>
-      <c r="J53" s="4" t="n"/>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M53" s="4" t="n"/>
       <c r="N53" s="4" t="n"/>
       <c r="O53" s="4" t="n"/>
@@ -4253,7 +4297,11 @@
       </c>
       <c r="H54" s="4" t="n"/>
       <c r="I54" s="4" t="n"/>
-      <c r="J54" s="4" t="n"/>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="M54" s="4" t="n"/>
       <c r="N54" s="4" t="n"/>
       <c r="O54" s="4" t="n"/>
@@ -4310,7 +4358,11 @@
       </c>
       <c r="H55" s="4" t="n"/>
       <c r="I55" s="4" t="n"/>
-      <c r="J55" s="4" t="n"/>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M55" s="4" t="n"/>
       <c r="N55" s="4" t="n"/>
       <c r="O55" s="4" t="n"/>
@@ -4365,7 +4417,11 @@
       </c>
       <c r="H56" s="4" t="n"/>
       <c r="I56" s="4" t="n"/>
-      <c r="J56" s="4" t="n"/>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M56" s="4" t="n"/>
       <c r="N56" s="4" t="n"/>
       <c r="O56" s="4" t="n"/>
@@ -4420,7 +4476,11 @@
       </c>
       <c r="H57" s="4" t="n"/>
       <c r="I57" s="4" t="n"/>
-      <c r="J57" s="4" t="n"/>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M57" s="4" t="n"/>
       <c r="N57" s="4" t="n"/>
       <c r="O57" s="4" t="n"/>
@@ -4476,7 +4536,11 @@
       </c>
       <c r="H58" s="4" t="n"/>
       <c r="I58" s="4" t="n"/>
-      <c r="J58" s="4" t="n"/>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M58" s="4" t="n"/>
       <c r="N58" s="4" t="n"/>
       <c r="O58" s="4" t="n"/>
@@ -4532,7 +4596,11 @@
       </c>
       <c r="H59" s="4" t="n"/>
       <c r="I59" s="4" t="n"/>
-      <c r="J59" s="4" t="n"/>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M59" s="4" t="n"/>
       <c r="N59" s="4" t="n"/>
       <c r="O59" s="4" t="n"/>
@@ -4587,7 +4655,11 @@
       </c>
       <c r="H60" s="4" t="n"/>
       <c r="I60" s="4" t="n"/>
-      <c r="J60" s="4" t="n"/>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="M60" s="4" t="n"/>
       <c r="N60" s="4" t="n"/>
       <c r="O60" s="4" t="n"/>
@@ -4643,7 +4715,11 @@
       </c>
       <c r="H61" s="4" t="n"/>
       <c r="I61" s="4" t="n"/>
-      <c r="J61" s="4" t="n"/>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M61" s="4" t="n"/>
       <c r="N61" s="4" t="n"/>
       <c r="O61" s="4" t="n"/>

</xml_diff>

<commit_message>
DeepSeek msgtxt run (18/19, 100% grounded)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -3638,7 +3638,11 @@
         </is>
       </c>
       <c r="H43" s="4" t="n"/>
-      <c r="I43" s="4" t="n"/>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -3698,7 +3702,11 @@
         </is>
       </c>
       <c r="H44" s="4" t="n"/>
-      <c r="I44" s="4" t="n"/>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -3758,7 +3766,11 @@
         </is>
       </c>
       <c r="H45" s="4" t="n"/>
-      <c r="I45" s="4" t="n"/>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -3817,7 +3829,11 @@
         </is>
       </c>
       <c r="H46" s="4" t="n"/>
-      <c r="I46" s="4" t="n"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="J46" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -3877,7 +3893,11 @@
         </is>
       </c>
       <c r="H47" s="4" t="n"/>
-      <c r="I47" s="4" t="n"/>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -3937,7 +3957,11 @@
         </is>
       </c>
       <c r="H48" s="4" t="n"/>
-      <c r="I48" s="4" t="n"/>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -3997,7 +4021,11 @@
         </is>
       </c>
       <c r="H49" s="4" t="n"/>
-      <c r="I49" s="4" t="n"/>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -4057,7 +4085,11 @@
         </is>
       </c>
       <c r="H50" s="4" t="n"/>
-      <c r="I50" s="4" t="n"/>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -4117,7 +4149,11 @@
         </is>
       </c>
       <c r="H51" s="4" t="n"/>
-      <c r="I51" s="4" t="n"/>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4176,7 +4212,11 @@
         </is>
       </c>
       <c r="H52" s="4" t="n"/>
-      <c r="I52" s="4" t="n"/>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -4237,7 +4277,11 @@
         </is>
       </c>
       <c r="H53" s="4" t="n"/>
-      <c r="I53" s="4" t="n"/>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4296,7 +4340,11 @@
         </is>
       </c>
       <c r="H54" s="4" t="n"/>
-      <c r="I54" s="4" t="n"/>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -4357,7 +4405,11 @@
         </is>
       </c>
       <c r="H55" s="4" t="n"/>
-      <c r="I55" s="4" t="n"/>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4416,7 +4468,11 @@
         </is>
       </c>
       <c r="H56" s="4" t="n"/>
-      <c r="I56" s="4" t="n"/>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4475,7 +4531,11 @@
         </is>
       </c>
       <c r="H57" s="4" t="n"/>
-      <c r="I57" s="4" t="n"/>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4535,7 +4595,11 @@
         </is>
       </c>
       <c r="H58" s="4" t="n"/>
-      <c r="I58" s="4" t="n"/>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="J58" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4595,7 +4659,11 @@
         </is>
       </c>
       <c r="H59" s="4" t="n"/>
-      <c r="I59" s="4" t="n"/>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="J59" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4654,7 +4722,11 @@
         </is>
       </c>
       <c r="H60" s="4" t="n"/>
-      <c r="I60" s="4" t="n"/>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -4714,7 +4786,11 @@
         </is>
       </c>
       <c r="H61" s="4" t="n"/>
-      <c r="I61" s="4" t="n"/>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="J61" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>

</xml_diff>

<commit_message>
Kimi msgtxt run (18/19); grounding check ignores leading speaker labels
- check_grounding.py: a fragment is grounded even if the model prepended a
  dialogue speaker label (e.g. 'Бека: ') to a mid-utterance quote (fixed 4
  false negatives in Kimi's msgtxt run -> 100% grounded)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -3648,6 +3648,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="M43" s="4" t="n"/>
       <c r="N43" s="4" t="n"/>
       <c r="O43" s="4" t="n"/>
@@ -3712,6 +3717,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="M44" s="4" t="n"/>
       <c r="N44" s="4" t="n"/>
       <c r="O44" s="4" t="n"/>
@@ -3776,6 +3786,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M45" s="4" t="n"/>
       <c r="N45" s="4" t="n"/>
       <c r="O45" s="4" t="n"/>
@@ -3839,6 +3854,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="M46" s="4" t="n"/>
       <c r="N46" s="4" t="n"/>
       <c r="O46" s="4" t="n"/>
@@ -3903,6 +3923,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M47" s="4" t="n"/>
       <c r="N47" s="4" t="n"/>
       <c r="O47" s="4" t="n"/>
@@ -3967,6 +3992,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M48" s="4" t="n"/>
       <c r="N48" s="4" t="n"/>
       <c r="O48" s="4" t="n"/>
@@ -4031,6 +4061,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="M49" s="4" t="n"/>
       <c r="N49" s="4" t="n"/>
       <c r="O49" s="4" t="n"/>
@@ -4095,6 +4130,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="M50" s="4" t="n"/>
       <c r="N50" s="4" t="n"/>
       <c r="O50" s="4" t="n"/>
@@ -4159,6 +4199,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M51" s="4" t="n"/>
       <c r="N51" s="4" t="n"/>
       <c r="O51" s="4" t="n"/>
@@ -4222,6 +4267,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="M52" s="4" t="n"/>
       <c r="N52" s="4" t="n"/>
       <c r="O52" s="4" t="n"/>
@@ -4287,6 +4337,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="M53" s="4" t="n"/>
       <c r="N53" s="4" t="n"/>
       <c r="O53" s="4" t="n"/>
@@ -4350,6 +4405,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="M54" s="4" t="n"/>
       <c r="N54" s="4" t="n"/>
       <c r="O54" s="4" t="n"/>
@@ -4415,6 +4475,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M55" s="4" t="n"/>
       <c r="N55" s="4" t="n"/>
       <c r="O55" s="4" t="n"/>
@@ -4478,6 +4543,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M56" s="4" t="n"/>
       <c r="N56" s="4" t="n"/>
       <c r="O56" s="4" t="n"/>
@@ -4541,6 +4611,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M57" s="4" t="n"/>
       <c r="N57" s="4" t="n"/>
       <c r="O57" s="4" t="n"/>
@@ -4605,6 +4680,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M58" s="4" t="n"/>
       <c r="N58" s="4" t="n"/>
       <c r="O58" s="4" t="n"/>
@@ -4669,6 +4749,11 @@
           <t>REFUTED</t>
         </is>
       </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="M59" s="4" t="n"/>
       <c r="N59" s="4" t="n"/>
       <c r="O59" s="4" t="n"/>
@@ -4732,6 +4817,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="M60" s="4" t="n"/>
       <c r="N60" s="4" t="n"/>
       <c r="O60" s="4" t="n"/>
@@ -4792,6 +4882,11 @@
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>

</xml_diff>

<commit_message>
Qwen msgtxt run (18/19, 100% grounded)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -3648,7 +3648,12 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K43" s="0" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -3717,7 +3722,12 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K44" s="0" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -3786,7 +3796,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K45" s="0" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -3854,7 +3869,12 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K46" s="0" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -3923,7 +3943,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K47" s="0" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -3992,7 +4017,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="K48" s="0" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4061,7 +4091,12 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="K49" s="0" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -4130,7 +4165,12 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="K50" s="0" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -4199,7 +4239,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
+      <c r="K51" s="0" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4267,7 +4312,12 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="K52" s="0" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -4337,7 +4387,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="K53" s="0" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -4405,7 +4460,12 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="K54" s="0" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -4475,7 +4535,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
+      <c r="K55" s="0" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4543,7 +4608,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="K56" s="0" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4611,7 +4681,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
+      <c r="K57" s="0" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4680,7 +4755,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
+      <c r="K58" s="0" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4749,7 +4829,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
+      <c r="K59" s="0" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4817,7 +4902,12 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
+      <c r="K60" s="0" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -4886,7 +4976,12 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
+      <c r="K61" s="0" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>

</xml_diff>

<commit_message>
Rework claim 052 into a clean causal inversion (fans<->concert)
- old 052 introduced 'traffic jams', a term absent from the dialogue, so the
  4 chat models correctly returned NEI (unsupported element), not a failed
  inversion. Reworded to invert only source-present elements (concert->fans).
- cleared stale chat-model 052 labels; marked chat msgtxt runs for re-run

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -3653,7 +3653,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L43" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -3727,7 +3727,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="L44" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -3801,7 +3801,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="L45" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -3874,7 +3874,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L46" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -3948,7 +3948,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
+      <c r="L47" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4022,7 +4022,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="L48" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4096,7 +4096,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="L49" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -4170,7 +4170,7 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr">
+      <c r="L50" s="0" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
         </is>
@@ -4244,7 +4244,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr">
+      <c r="L51" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4317,7 +4317,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr">
+      <c r="L52" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -4357,7 +4357,7 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Алматыда кептелістер салдарынан Скриптониттің концерті өтетін болады</t>
+          <t>Алматыда фанаттар көп жиналатындықтан, Скриптониттің концерті өтетін болады.</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
@@ -4367,8 +4367,7 @@
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Скриптонит қой, полный живой звук болады деді. Прикинь в ате толпа фанатов наверное будет, бакад аман болсын.
-</t>
+          <t>Себеп-салдар инверсиясы: концерт→фанаттар (түпнұсқа) орнына фанаттар→концерт</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -4377,26 +4376,14 @@
         </is>
       </c>
       <c r="H53" s="4" t="n"/>
-      <c r="I53" s="4" t="inlineStr">
-        <is>
-          <t>NOT_ENOUGH_INFO</t>
-        </is>
-      </c>
+      <c r="I53" s="4" t="n"/>
       <c r="J53" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K53" s="0" t="inlineStr">
-        <is>
-          <t>NOT_ENOUGH_INFO</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>NOT_ENOUGH_INFO</t>
-        </is>
-      </c>
+      <c r="K53" s="0" t="n"/>
+      <c r="L53" s="0" t="n"/>
       <c r="M53" s="4" t="n"/>
       <c r="N53" s="4" t="n"/>
       <c r="O53" s="4" t="n"/>
@@ -4465,7 +4452,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr">
+      <c r="L54" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -4540,7 +4527,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr">
+      <c r="L55" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4613,7 +4600,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L56" t="inlineStr">
+      <c r="L56" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4686,7 +4673,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr">
+      <c r="L57" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4760,7 +4747,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L58" t="inlineStr">
+      <c r="L58" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4834,7 +4821,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L59" t="inlineStr">
+      <c r="L59" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
@@ -4907,7 +4894,7 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="L60" t="inlineStr">
+      <c r="L60" s="0" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
         </is>
@@ -4981,7 +4968,7 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L61" t="inlineStr">
+      <c r="L61" s="0" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>

</xml_diff>

<commit_message>
Re-run DeepSeek & Kimi on corrected 052
- DeepSeek still NEI on the clean inversion (genuine causal weakness): 18/19
- Kimi caught it (REFUTED/causal): 19/19

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -4376,13 +4376,21 @@
         </is>
       </c>
       <c r="H53" s="4" t="n"/>
-      <c r="I53" s="4" t="n"/>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="K53" s="0" t="n"/>
+      <c r="K53" s="0" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="L53" s="0" t="n"/>
       <c r="M53" s="4" t="n"/>
       <c r="N53" s="4" t="n"/>

</xml_diff>

<commit_message>
Re-run Qwen on corrected 052 (still NEI): 18/19
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -4391,7 +4391,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="L53" s="0" t="n"/>
+      <c r="L53" s="0" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="M53" s="4" t="n"/>
       <c r="N53" s="4" t="n"/>
       <c r="O53" s="4" t="n"/>

</xml_diff>

<commit_message>
Add Gemini msgtxt run (19/19) + backfill Gemini news evidence — 60 claims x 5 models complete
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bHj5cjv4Bcvyqx2j9qjtM
</commit_message>
<xml_diff>
--- a/factcheck_dataset.xlsx
+++ b/factcheck_dataset.xlsx
@@ -3637,7 +3637,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H43" s="4" t="n"/>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -3711,7 +3715,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H44" s="4" t="n"/>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -3785,7 +3793,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H45" s="4" t="n"/>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -3858,7 +3870,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="H46" s="4" t="n"/>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -3932,7 +3948,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H47" s="4" t="n"/>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4006,7 +4026,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H48" s="4" t="n"/>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4080,7 +4104,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H49" s="4" t="n"/>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -4154,7 +4182,11 @@
           <t>SUPPORTED</t>
         </is>
       </c>
-      <c r="H50" s="4" t="n"/>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>SUPPORTED</t>
+        </is>
+      </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
           <t>SUPPORTED</t>
@@ -4228,7 +4260,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H51" s="4" t="n"/>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4301,7 +4337,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="H52" s="4" t="n"/>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -4375,7 +4415,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H53" s="4" t="n"/>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -4448,7 +4492,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="H54" s="4" t="n"/>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -4523,7 +4571,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H55" s="4" t="n"/>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4596,7 +4648,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H56" s="4" t="n"/>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4669,7 +4725,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H57" s="4" t="n"/>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4743,7 +4803,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H58" s="4" t="n"/>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4817,7 +4881,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H59" s="4" t="n"/>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>
@@ -4890,7 +4958,11 @@
           <t>NOT_ENOUGH_INFO</t>
         </is>
       </c>
-      <c r="H60" s="4" t="n"/>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>NOT_ENOUGH_INFO</t>
+        </is>
+      </c>
       <c r="I60" s="4" t="inlineStr">
         <is>
           <t>NOT_ENOUGH_INFO</t>
@@ -4964,7 +5036,11 @@
           <t>REFUTED</t>
         </is>
       </c>
-      <c r="H61" s="4" t="n"/>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED</t>
+        </is>
+      </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
           <t>REFUTED</t>

</xml_diff>